<commit_message>
Excel table is now final. Added regression over interaction term with help, but no clear results.
</commit_message>
<xml_diff>
--- a/evaluation/AMLTA Experiment.xlsx
+++ b/evaluation/AMLTA Experiment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\am200\OneDrive\Desktop\AMLFTA\DrivingCoachRepo\DrivingCoach\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67303559-9002-4583-B9A1-E5C98DA381B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1A3135-A5BA-4EA7-BE58-C5C9016C2A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E8119279-4CFB-428F-BC2B-7CF76D7BCF0B}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="85">
   <si>
     <t>EXPERIMENT - RACE</t>
   </si>
@@ -85,10 +85,31 @@
     <t>Erfahrung</t>
   </si>
   <si>
-    <t>Hilfe</t>
+    <t>name</t>
   </si>
   <si>
-    <t>Gesamtdauer</t>
+    <t>id</t>
+  </si>
+  <si>
+    <t>racetrack</t>
+  </si>
+  <si>
+    <t>help</t>
+  </si>
+  <si>
+    <t>experience</t>
+  </si>
+  <si>
+    <t>total_duration</t>
+  </si>
+  <si>
+    <t>lap</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>Hilfe</t>
   </si>
   <si>
     <t>AmL ID5</t>
@@ -125,6 +146,9 @@
   </si>
   <si>
     <t>LM ID21</t>
+  </si>
+  <si>
+    <t>VG ID23</t>
   </si>
   <si>
     <t>LW ID1</t>
@@ -166,10 +190,10 @@
     <t>FW ID22</t>
   </si>
   <si>
-    <t>In der DB fehlend</t>
+    <t>ES</t>
   </si>
   <si>
-    <t>In der BC unter dem Kürzel von lennard</t>
+    <t>fehlt</t>
   </si>
   <si>
     <t>Ohne hilfe</t>
@@ -209,6 +233,9 @@
   </si>
   <si>
     <t>Welche Strecke</t>
+  </si>
+  <si>
+    <t>Gesamtdauer</t>
   </si>
   <si>
     <t>Kart: Produkt (nachher nicht in den Datensatz einfügen!)</t>
@@ -289,31 +316,7 @@
     <t>Etienne</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>racetrack</t>
-  </si>
-  <si>
-    <t>experience</t>
-  </si>
-  <si>
-    <t>lap</t>
-  </si>
-  <si>
-    <t>duration</t>
-  </si>
-  <si>
-    <t>total_duration</t>
-  </si>
-  <si>
     <t>race_number</t>
-  </si>
-  <si>
-    <t>help</t>
   </si>
 </sst>
 </file>
@@ -486,17 +489,7 @@
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color theme="1"/>
@@ -892,17 +885,13 @@
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.5703125" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="11.5703125" customWidth="1"/>
     <col min="25" max="25" width="2.42578125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="1.42578125" customWidth="1"/>
@@ -975,52 +964,52 @@
         <v>6</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="S5" s="8" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="Y5" s="8"/>
       <c r="Z5" s="8"/>
@@ -1033,7 +1022,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
@@ -1093,13 +1082,13 @@
         <v>60</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="Y6">
         <v>1</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
@@ -1107,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -1160,19 +1149,19 @@
         <v>1</v>
       </c>
       <c r="T7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U7" s="15">
         <v>60</v>
       </c>
       <c r="X7" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="Y7">
         <v>2</v>
       </c>
       <c r="AA7" s="3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
@@ -1180,7 +1169,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
@@ -1233,20 +1222,20 @@
         <v>1</v>
       </c>
       <c r="T8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U8" s="12">
         <v>74.42</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Y8" s="5">
         <v>3</v>
       </c>
       <c r="Z8" s="5"/>
       <c r="AA8" s="6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
@@ -1254,7 +1243,7 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3">
         <v>1</v>
@@ -1318,7 +1307,7 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
@@ -1371,7 +1360,7 @@
         <v>1</v>
       </c>
       <c r="T10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U10" s="12">
         <v>62.13</v>
@@ -1382,7 +1371,7 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C11" s="3">
         <v>1</v>
@@ -1435,7 +1424,7 @@
         <v>1</v>
       </c>
       <c r="T11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U11" s="12">
         <v>131.52000000000001</v>
@@ -1445,6 +1434,9 @@
       <c r="A12" s="2">
         <v>7</v>
       </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
       <c r="C12" s="3">
         <v>1</v>
       </c>
@@ -1496,7 +1488,7 @@
         <v>1</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U12" s="12">
         <v>92.23</v>
@@ -1507,7 +1499,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C13" s="3">
         <v>2</v>
@@ -1571,7 +1563,7 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C14" s="3">
         <v>2</v>
@@ -1624,7 +1616,7 @@
         <v>1</v>
       </c>
       <c r="T14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="12">
         <v>80.48</v>
@@ -1636,7 +1628,7 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C15" s="3">
         <v>2</v>
@@ -1689,7 +1681,7 @@
         <v>1</v>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U15" s="12">
         <v>103</v>
@@ -1700,7 +1692,7 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C16" s="3">
         <v>2</v>
@@ -1753,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="T16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" s="12">
         <v>100.24</v>
@@ -1764,7 +1756,7 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C17" s="3">
         <v>2</v>
@@ -1828,7 +1820,7 @@
         <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C18" s="3">
         <v>2</v>
@@ -1881,7 +1873,7 @@
         <v>1</v>
       </c>
       <c r="T18">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U18" s="12">
         <v>96.22</v>
@@ -1892,7 +1884,7 @@
         <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C19" s="3">
         <v>2</v>
@@ -1945,7 +1937,7 @@
         <v>1</v>
       </c>
       <c r="T19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U19" s="12">
         <v>90.83</v>
@@ -1956,7 +1948,7 @@
         <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C20" s="3">
         <v>3</v>
@@ -2020,7 +2012,7 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C21" s="3">
         <v>3</v>
@@ -2084,7 +2076,7 @@
         <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C22" s="3">
         <v>3</v>
@@ -2137,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="T22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U22" s="12">
         <v>84.65</v>
@@ -2148,7 +2140,7 @@
         <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C23" s="3">
         <v>3</v>
@@ -2201,7 +2193,7 @@
         <v>1</v>
       </c>
       <c r="T23">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U23" s="12">
         <v>80.349999999999994</v>
@@ -2212,14 +2204,14 @@
         <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C24" s="3">
         <v>3</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="F24">
         <v>7</v>
@@ -2238,7 +2230,7 @@
       </c>
       <c r="K24" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>589.67999999999995</v>
       </c>
       <c r="N24" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2276,14 +2268,14 @@
         <v>20</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C25" s="3">
         <v>3</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="F25">
         <v>7</v>
@@ -2302,7 +2294,7 @@
       </c>
       <c r="K25" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>419.93999999999994</v>
       </c>
       <c r="N25" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2329,7 +2321,7 @@
         <v>1</v>
       </c>
       <c r="T25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U25" s="12">
         <v>112.42</v>
@@ -2339,13 +2331,15 @@
       <c r="A26" s="4">
         <v>21</v>
       </c>
-      <c r="B26" s="5"/>
+      <c r="B26" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="C26" s="6">
         <v>3</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="F26">
         <v>7</v>
@@ -2364,7 +2358,7 @@
       </c>
       <c r="K26" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>524.63</v>
       </c>
       <c r="N26" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2391,7 +2385,7 @@
         <v>1</v>
       </c>
       <c r="T26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U26" s="12">
         <v>95.34</v>
@@ -2446,7 +2440,7 @@
         <v>1</v>
       </c>
       <c r="T27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U27" s="12">
         <v>112.21</v>
@@ -2556,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="T29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U29" s="12">
         <v>97.75</v>
@@ -2611,7 +2605,7 @@
         <v>1</v>
       </c>
       <c r="T30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U30" s="12">
         <v>84.55</v>
@@ -2666,7 +2660,7 @@
         <v>1</v>
       </c>
       <c r="T31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U31" s="12">
         <v>62.06</v>
@@ -2776,7 +2770,7 @@
         <v>1</v>
       </c>
       <c r="T33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U33" s="12">
         <v>63.09</v>
@@ -2831,7 +2825,7 @@
         <v>1</v>
       </c>
       <c r="T34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U34" s="12">
         <v>63.75</v>
@@ -2996,7 +2990,7 @@
         <v>1</v>
       </c>
       <c r="T37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U37" s="12">
         <v>97.53</v>
@@ -3051,7 +3045,7 @@
         <v>1</v>
       </c>
       <c r="T38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U38" s="12">
         <v>109.34</v>
@@ -3161,7 +3155,7 @@
         <v>1</v>
       </c>
       <c r="T40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U40" s="12">
         <v>69.69</v>
@@ -3216,7 +3210,7 @@
         <v>1</v>
       </c>
       <c r="T41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U41" s="12">
         <v>72.12</v>
@@ -3271,7 +3265,7 @@
         <v>1</v>
       </c>
       <c r="T42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U42" s="12">
         <v>63.04</v>
@@ -3381,7 +3375,7 @@
         <v>1</v>
       </c>
       <c r="T44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U44" s="12">
         <v>54.28</v>
@@ -3436,7 +3430,7 @@
         <v>1</v>
       </c>
       <c r="T45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U45" s="12">
         <v>55.54</v>
@@ -3491,7 +3485,7 @@
         <v>1</v>
       </c>
       <c r="T46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U46" s="12">
         <v>106.94</v>
@@ -3601,7 +3595,7 @@
         <v>1</v>
       </c>
       <c r="T48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U48" s="12">
         <v>87.44</v>
@@ -3656,7 +3650,7 @@
         <v>1</v>
       </c>
       <c r="T49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U49" s="12">
         <v>80.5</v>
@@ -3821,7 +3815,7 @@
         <v>1</v>
       </c>
       <c r="T52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U52">
         <v>78.760000000000005</v>
@@ -3849,7 +3843,7 @@
       </c>
       <c r="K53" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>293.83999999999997</v>
       </c>
       <c r="N53" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3876,7 +3870,7 @@
         <v>1</v>
       </c>
       <c r="T53">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U53">
         <v>81.099999999999994</v>
@@ -3986,7 +3980,7 @@
         <v>1</v>
       </c>
       <c r="T55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U55">
         <v>78.78</v>
@@ -4041,7 +4035,7 @@
         <v>1</v>
       </c>
       <c r="T56">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U56" s="15">
         <v>73.510000000000005</v>
@@ -4096,7 +4090,7 @@
         <v>1</v>
       </c>
       <c r="T57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U57" s="15">
         <v>73.67</v>
@@ -4206,7 +4200,7 @@
         <v>1</v>
       </c>
       <c r="T59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U59" s="15">
         <v>72.03</v>
@@ -4261,7 +4255,7 @@
         <v>1</v>
       </c>
       <c r="T60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U60" s="15">
         <v>68.17</v>
@@ -4316,7 +4310,7 @@
         <v>1</v>
       </c>
       <c r="T61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U61">
         <v>53.79</v>
@@ -4426,7 +4420,7 @@
         <v>1</v>
       </c>
       <c r="T63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U63">
         <v>50.58</v>
@@ -4481,7 +4475,7 @@
         <v>1</v>
       </c>
       <c r="T64">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U64">
         <v>60.08</v>
@@ -4543,9 +4537,9 @@
       </c>
     </row>
     <row r="66" spans="5:21" x14ac:dyDescent="0.25">
-      <c r="E66" s="2">
+      <c r="E66" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="F66">
         <v>21</v>
@@ -4564,7 +4558,7 @@
       </c>
       <c r="K66" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>308.27999999999997</v>
       </c>
       <c r="N66" s="2" t="str">
         <f t="shared" si="2"/>
@@ -4598,9 +4592,9 @@
       </c>
     </row>
     <row r="67" spans="5:21" x14ac:dyDescent="0.25">
-      <c r="E67" s="2">
+      <c r="E67" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="F67">
         <v>21</v>
@@ -4619,7 +4613,7 @@
       </c>
       <c r="K67" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>283.51000000000005</v>
       </c>
       <c r="N67" s="2" t="str">
         <f t="shared" si="2"/>
@@ -4646,16 +4640,16 @@
         <v>1</v>
       </c>
       <c r="T67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U67" s="12">
         <v>91.99</v>
       </c>
     </row>
     <row r="68" spans="5:21" x14ac:dyDescent="0.25">
-      <c r="E68" s="4">
+      <c r="E68" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="F68" s="5">
         <v>21</v>
@@ -4674,7 +4668,7 @@
       </c>
       <c r="K68" s="12">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>212.26999999999998</v>
       </c>
       <c r="N68" s="2" t="str">
         <f t="shared" si="2"/>
@@ -4700,8 +4694,8 @@
         <f t="array" ref="S68">INDEX($I$6:$I$68, INT((ROWS(S$6:S68)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="T68" s="5">
-        <v>3</v>
+      <c r="T68">
+        <v>1</v>
       </c>
       <c r="U68" s="12">
         <v>83.75</v>
@@ -4732,6 +4726,9 @@
         <f t="array" ref="S69">INDEX($I$6:$I$68, INT((ROWS(S$6:S69)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T69">
+        <v>1</v>
+      </c>
       <c r="U69" s="12">
         <v>102.53</v>
       </c>
@@ -4761,6 +4758,9 @@
         <f t="array" ref="S70">INDEX($I$6:$I$68, INT((ROWS(S$6:S70)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T70">
+        <v>1</v>
+      </c>
       <c r="U70" s="12">
         <v>108.59</v>
       </c>
@@ -4790,6 +4790,9 @@
         <f t="array" ref="S71">INDEX($I$6:$I$68, INT((ROWS(S$6:S71)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T71">
+        <v>2</v>
+      </c>
       <c r="U71" s="12">
         <v>76.209999999999994</v>
       </c>
@@ -4819,6 +4822,9 @@
         <f t="array" ref="S72">INDEX($I$6:$I$68, INT((ROWS(S$6:S72)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T72">
+        <v>2</v>
+      </c>
       <c r="U72" s="12">
         <v>61.1</v>
       </c>
@@ -4848,6 +4854,9 @@
         <f t="array" ref="S73">INDEX($I$6:$I$68, INT((ROWS(S$6:S73)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T73">
+        <v>2</v>
+      </c>
       <c r="U73" s="12">
         <v>59.02</v>
       </c>
@@ -4877,6 +4886,9 @@
         <f t="array" ref="S74">INDEX($I$6:$I$68, INT((ROWS(S$6:S74)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T74">
+        <v>2</v>
+      </c>
       <c r="U74" s="12">
         <v>79.069999999999993</v>
       </c>
@@ -4906,6 +4918,9 @@
         <f t="array" ref="S75">INDEX($I$6:$I$68, INT((ROWS(S$6:S75)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T75">
+        <v>2</v>
+      </c>
       <c r="U75" s="12">
         <v>56.8</v>
       </c>
@@ -4935,6 +4950,9 @@
         <f t="array" ref="S76">INDEX($I$6:$I$68, INT((ROWS(S$6:S76)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T76">
+        <v>3</v>
+      </c>
       <c r="U76" s="12">
         <v>81.099999999999994</v>
       </c>
@@ -4964,6 +4982,9 @@
         <f t="array" ref="S77">INDEX($I$6:$I$68, INT((ROWS(S$6:S77)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T77">
+        <v>3</v>
+      </c>
       <c r="U77" s="12">
         <v>79.55</v>
       </c>
@@ -4993,6 +5014,9 @@
         <f t="array" ref="S78">INDEX($I$6:$I$68, INT((ROWS(S$6:S78)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T78">
+        <v>3</v>
+      </c>
       <c r="U78" s="12">
         <v>75.52</v>
       </c>
@@ -5022,6 +5046,9 @@
         <f t="array" ref="S79">INDEX($I$6:$I$68, INT((ROWS(S$6:S79)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T79">
+        <v>3</v>
+      </c>
       <c r="U79" s="12">
         <v>74.760000000000005</v>
       </c>
@@ -5051,6 +5078,9 @@
         <f t="array" ref="S80">INDEX($I$6:$I$68, INT((ROWS(S$6:S80)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T80">
+        <v>3</v>
+      </c>
       <c r="U80" s="12">
         <v>81.650000000000006</v>
       </c>
@@ -5080,6 +5110,9 @@
         <f t="array" ref="S81">INDEX($I$6:$I$68, INT((ROWS(S$6:S81)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T81">
+        <v>1</v>
+      </c>
       <c r="U81" s="12">
         <v>69.36</v>
       </c>
@@ -5109,6 +5142,9 @@
         <f t="array" ref="S82">INDEX($I$6:$I$68, INT((ROWS(S$6:S82)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T82">
+        <v>1</v>
+      </c>
       <c r="U82" s="12">
         <v>55.63</v>
       </c>
@@ -5138,6 +5174,9 @@
         <f t="array" ref="S83">INDEX($I$6:$I$68, INT((ROWS(S$6:S83)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T83">
+        <v>1</v>
+      </c>
       <c r="U83" s="12">
         <v>64.569999999999993</v>
       </c>
@@ -5167,6 +5206,9 @@
         <f t="array" ref="S84">INDEX($I$6:$I$68, INT((ROWS(S$6:S84)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T84">
+        <v>1</v>
+      </c>
       <c r="U84" s="12">
         <v>51.03</v>
       </c>
@@ -5196,6 +5238,9 @@
         <f t="array" ref="S85">INDEX($I$6:$I$68, INT((ROWS(S$6:S85)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T85">
+        <v>1</v>
+      </c>
       <c r="U85" s="12">
         <v>55.76</v>
       </c>
@@ -5225,6 +5270,9 @@
         <f t="array" ref="S86">INDEX($I$6:$I$68, INT((ROWS(S$6:S86)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T86">
+        <v>2</v>
+      </c>
       <c r="U86" s="12">
         <v>85</v>
       </c>
@@ -5255,6 +5303,9 @@
         <f t="array" ref="S87">INDEX($I$6:$I$68, INT((ROWS(S$6:S87)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T87">
+        <v>2</v>
+      </c>
       <c r="U87" s="12">
         <v>94.19</v>
       </c>
@@ -5285,6 +5336,9 @@
         <f t="array" ref="S88">INDEX($I$6:$I$68, INT((ROWS(S$6:S88)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T88">
+        <v>2</v>
+      </c>
       <c r="U88" s="12">
         <f>6+60+18</f>
         <v>84</v>
@@ -5316,6 +5370,9 @@
         <f t="array" ref="S89">INDEX($I$6:$I$68, INT((ROWS(S$6:S89)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T89">
+        <v>2</v>
+      </c>
       <c r="U89" s="12">
         <v>92.41</v>
       </c>
@@ -5345,6 +5402,9 @@
         <f t="array" ref="S90">INDEX($I$6:$I$68, INT((ROWS(S$6:S90)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T90">
+        <v>2</v>
+      </c>
       <c r="U90" s="12">
         <v>66.19</v>
       </c>
@@ -5374,6 +5434,9 @@
         <f t="array" ref="S91">INDEX($I$6:$I$68, INT((ROWS(S$6:S91)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T91">
+        <v>3</v>
+      </c>
       <c r="U91">
         <v>74.36</v>
       </c>
@@ -5404,6 +5467,9 @@
         <f t="array" ref="S92">INDEX($I$6:$I$68, INT((ROWS(S$6:S92)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T92">
+        <v>3</v>
+      </c>
       <c r="U92">
         <v>93</v>
       </c>
@@ -5433,6 +5499,9 @@
         <f t="array" ref="S93">INDEX($I$6:$I$68, INT((ROWS(S$6:S93)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T93">
+        <v>3</v>
+      </c>
       <c r="U93" s="12">
         <v>87.63</v>
       </c>
@@ -5462,6 +5531,9 @@
         <f t="array" ref="S94">INDEX($I$6:$I$68, INT((ROWS(S$6:S94)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T94">
+        <v>3</v>
+      </c>
       <c r="U94" s="12">
         <v>92.89</v>
       </c>
@@ -5491,14 +5563,17 @@
         <f t="array" ref="S95">INDEX($I$6:$I$68, INT((ROWS(S$6:S95)-1)/5)+1)</f>
         <v>1</v>
       </c>
+      <c r="T95">
+        <v>3</v>
+      </c>
       <c r="U95" s="12">
         <v>73</v>
       </c>
     </row>
     <row r="96" spans="14:24" x14ac:dyDescent="0.25">
-      <c r="N96" s="2">
+      <c r="N96" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O96" cm="1">
         <f t="array" ref="O96">INDEX($F$6:$F$68, INT((ROWS(O$6:O96)-1)/5)+1)</f>
@@ -5520,12 +5595,17 @@
         <f t="array" ref="S96">INDEX($I$6:$I$68, INT((ROWS(S$6:S96)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U96" s="12"/>
+      <c r="T96">
+        <v>1</v>
+      </c>
+      <c r="U96" s="12">
+        <v>121.86</v>
+      </c>
     </row>
     <row r="97" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N97" s="2">
+      <c r="N97" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O97" cm="1">
         <f t="array" ref="O97">INDEX($F$6:$F$68, INT((ROWS(O$6:O97)-1)/5)+1)</f>
@@ -5547,12 +5627,17 @@
         <f t="array" ref="S97">INDEX($I$6:$I$68, INT((ROWS(S$6:S97)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U97" s="12"/>
+      <c r="T97">
+        <v>1</v>
+      </c>
+      <c r="U97" s="12">
+        <v>123.42</v>
+      </c>
     </row>
     <row r="98" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N98" s="2">
+      <c r="N98" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O98" cm="1">
         <f t="array" ref="O98">INDEX($F$6:$F$68, INT((ROWS(O$6:O98)-1)/5)+1)</f>
@@ -5574,12 +5659,17 @@
         <f t="array" ref="S98">INDEX($I$6:$I$68, INT((ROWS(S$6:S98)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U98" s="12"/>
+      <c r="T98">
+        <v>1</v>
+      </c>
+      <c r="U98" s="12">
+        <v>129.37</v>
+      </c>
     </row>
     <row r="99" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N99" s="2">
+      <c r="N99" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O99" cm="1">
         <f t="array" ref="O99">INDEX($F$6:$F$68, INT((ROWS(O$6:O99)-1)/5)+1)</f>
@@ -5601,12 +5691,17 @@
         <f t="array" ref="S99">INDEX($I$6:$I$68, INT((ROWS(S$6:S99)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U99" s="12"/>
+      <c r="T99">
+        <v>1</v>
+      </c>
+      <c r="U99" s="12">
+        <v>104.87</v>
+      </c>
     </row>
     <row r="100" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N100" s="2">
+      <c r="N100" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O100" cm="1">
         <f t="array" ref="O100">INDEX($F$6:$F$68, INT((ROWS(O$6:O100)-1)/5)+1)</f>
@@ -5628,12 +5723,17 @@
         <f t="array" ref="S100">INDEX($I$6:$I$68, INT((ROWS(S$6:S100)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U100" s="12"/>
+      <c r="T100">
+        <v>1</v>
+      </c>
+      <c r="U100" s="12">
+        <v>110.16</v>
+      </c>
     </row>
     <row r="101" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N101" s="2">
+      <c r="N101" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O101" cm="1">
         <f t="array" ref="O101">INDEX($F$6:$F$68, INT((ROWS(O$6:O101)-1)/5)+1)</f>
@@ -5655,12 +5755,17 @@
         <f t="array" ref="S101">INDEX($I$6:$I$68, INT((ROWS(S$6:S101)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U101" s="12"/>
+      <c r="T101">
+        <v>2</v>
+      </c>
+      <c r="U101" s="12">
+        <v>76.38</v>
+      </c>
     </row>
     <row r="102" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N102" s="2">
+      <c r="N102" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O102" cm="1">
         <f t="array" ref="O102">INDEX($F$6:$F$68, INT((ROWS(O$6:O102)-1)/5)+1)</f>
@@ -5682,12 +5787,17 @@
         <f t="array" ref="S102">INDEX($I$6:$I$68, INT((ROWS(S$6:S102)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U102" s="12"/>
+      <c r="T102">
+        <v>2</v>
+      </c>
+      <c r="U102" s="12">
+        <v>86.87</v>
+      </c>
     </row>
     <row r="103" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N103" s="2">
+      <c r="N103" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O103" cm="1">
         <f t="array" ref="O103">INDEX($F$6:$F$68, INT((ROWS(O$6:O103)-1)/5)+1)</f>
@@ -5709,12 +5819,17 @@
         <f t="array" ref="S103">INDEX($I$6:$I$68, INT((ROWS(S$6:S103)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U103" s="12"/>
+      <c r="T103">
+        <v>2</v>
+      </c>
+      <c r="U103" s="12">
+        <v>95.33</v>
+      </c>
     </row>
     <row r="104" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N104" s="2">
+      <c r="N104" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O104" cm="1">
         <f t="array" ref="O104">INDEX($F$6:$F$68, INT((ROWS(O$6:O104)-1)/5)+1)</f>
@@ -5736,12 +5851,17 @@
         <f t="array" ref="S104">INDEX($I$6:$I$68, INT((ROWS(S$6:S104)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U104" s="12"/>
+      <c r="T104">
+        <v>2</v>
+      </c>
+      <c r="U104" s="12">
+        <v>77.47</v>
+      </c>
     </row>
     <row r="105" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N105" s="2">
+      <c r="N105" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O105" cm="1">
         <f t="array" ref="O105">INDEX($F$6:$F$68, INT((ROWS(O$6:O105)-1)/5)+1)</f>
@@ -5763,12 +5883,17 @@
         <f t="array" ref="S105">INDEX($I$6:$I$68, INT((ROWS(S$6:S105)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U105" s="12"/>
+      <c r="T105">
+        <v>2</v>
+      </c>
+      <c r="U105" s="12">
+        <v>83.89</v>
+      </c>
     </row>
     <row r="106" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N106" s="2">
+      <c r="N106" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O106" cm="1">
         <f t="array" ref="O106">INDEX($F$6:$F$68, INT((ROWS(O$6:O106)-1)/5)+1)</f>
@@ -5790,12 +5915,17 @@
         <f t="array" ref="S106">INDEX($I$6:$I$68, INT((ROWS(S$6:S106)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U106" s="12"/>
+      <c r="T106">
+        <v>3</v>
+      </c>
+      <c r="U106" s="12">
+        <v>110.14</v>
+      </c>
     </row>
     <row r="107" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N107" s="2">
+      <c r="N107" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O107" cm="1">
         <f t="array" ref="O107">INDEX($F$6:$F$68, INT((ROWS(O$6:O107)-1)/5)+1)</f>
@@ -5817,12 +5947,17 @@
         <f t="array" ref="S107">INDEX($I$6:$I$68, INT((ROWS(S$6:S107)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U107" s="12"/>
+      <c r="T107">
+        <v>3</v>
+      </c>
+      <c r="U107" s="12">
+        <v>103.67</v>
+      </c>
     </row>
     <row r="108" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N108" s="2">
+      <c r="N108" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O108" cm="1">
         <f t="array" ref="O108">INDEX($F$6:$F$68, INT((ROWS(O$6:O108)-1)/5)+1)</f>
@@ -5844,12 +5979,17 @@
         <f t="array" ref="S108">INDEX($I$6:$I$68, INT((ROWS(S$6:S108)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U108" s="12"/>
+      <c r="T108">
+        <v>3</v>
+      </c>
+      <c r="U108" s="12">
+        <v>108.93</v>
+      </c>
     </row>
     <row r="109" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N109" s="2">
+      <c r="N109" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O109" cm="1">
         <f t="array" ref="O109">INDEX($F$6:$F$68, INT((ROWS(O$6:O109)-1)/5)+1)</f>
@@ -5871,12 +6011,17 @@
         <f t="array" ref="S109">INDEX($I$6:$I$68, INT((ROWS(S$6:S109)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U109" s="12"/>
+      <c r="T109">
+        <v>3</v>
+      </c>
+      <c r="U109" s="12">
+        <v>99.51</v>
+      </c>
     </row>
     <row r="110" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N110" s="2">
+      <c r="N110" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>VG ID23</v>
       </c>
       <c r="O110" cm="1">
         <f t="array" ref="O110">INDEX($F$6:$F$68, INT((ROWS(O$6:O110)-1)/5)+1)</f>
@@ -5898,7 +6043,12 @@
         <f t="array" ref="S110">INDEX($I$6:$I$68, INT((ROWS(S$6:S110)-1)/5)+1)</f>
         <v>1</v>
       </c>
-      <c r="U110" s="12"/>
+      <c r="T110">
+        <v>3</v>
+      </c>
+      <c r="U110" s="12">
+        <v>102.38</v>
+      </c>
     </row>
     <row r="111" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N111" s="2" t="str">
@@ -5925,6 +6075,9 @@
         <f t="array" ref="S111">INDEX($I$6:$I$68, INT((ROWS(S$6:S111)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T111">
+        <v>1</v>
+      </c>
       <c r="U111" s="12">
         <v>58.04</v>
       </c>
@@ -5954,6 +6107,9 @@
         <f t="array" ref="S112">INDEX($I$6:$I$68, INT((ROWS(S$6:S112)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T112">
+        <v>1</v>
+      </c>
       <c r="U112" s="12">
         <v>52.75</v>
       </c>
@@ -5983,6 +6139,9 @@
         <f t="array" ref="S113">INDEX($I$6:$I$68, INT((ROWS(S$6:S113)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T113">
+        <v>1</v>
+      </c>
       <c r="U113" s="12">
         <v>51.5</v>
       </c>
@@ -6012,6 +6171,9 @@
         <f t="array" ref="S114">INDEX($I$6:$I$68, INT((ROWS(S$6:S114)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T114">
+        <v>1</v>
+      </c>
       <c r="U114" s="12">
         <v>51.75</v>
       </c>
@@ -6041,6 +6203,9 @@
         <f t="array" ref="S115">INDEX($I$6:$I$68, INT((ROWS(S$6:S115)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T115">
+        <v>1</v>
+      </c>
       <c r="U115" s="12">
         <v>55.44</v>
       </c>
@@ -6070,6 +6235,9 @@
         <f t="array" ref="S116">INDEX($I$6:$I$68, INT((ROWS(S$6:S116)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T116">
+        <v>2</v>
+      </c>
       <c r="U116" s="12">
         <v>80.58</v>
       </c>
@@ -6099,6 +6267,9 @@
         <f t="array" ref="S117">INDEX($I$6:$I$68, INT((ROWS(S$6:S117)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T117">
+        <v>2</v>
+      </c>
       <c r="U117" s="12">
         <v>98.35</v>
       </c>
@@ -6128,6 +6299,9 @@
         <f t="array" ref="S118">INDEX($I$6:$I$68, INT((ROWS(S$6:S118)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T118">
+        <v>2</v>
+      </c>
       <c r="U118" s="12">
         <v>77.61</v>
       </c>
@@ -6157,6 +6331,9 @@
         <f t="array" ref="S119">INDEX($I$6:$I$68, INT((ROWS(S$6:S119)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T119">
+        <v>2</v>
+      </c>
       <c r="U119" s="12">
         <v>77.959999999999994</v>
       </c>
@@ -6186,6 +6363,9 @@
         <f t="array" ref="S120">INDEX($I$6:$I$68, INT((ROWS(S$6:S120)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T120">
+        <v>2</v>
+      </c>
       <c r="U120" s="12">
         <v>71.319999999999993</v>
       </c>
@@ -6215,6 +6395,9 @@
         <f t="array" ref="S121">INDEX($I$6:$I$68, INT((ROWS(S$6:S121)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T121">
+        <v>3</v>
+      </c>
       <c r="U121" s="12">
         <v>65.88</v>
       </c>
@@ -6244,6 +6427,9 @@
         <f t="array" ref="S122">INDEX($I$6:$I$68, INT((ROWS(S$6:S122)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T122">
+        <v>3</v>
+      </c>
       <c r="U122" s="12">
         <v>62.23</v>
       </c>
@@ -6273,6 +6459,9 @@
         <f t="array" ref="S123">INDEX($I$6:$I$68, INT((ROWS(S$6:S123)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T123">
+        <v>3</v>
+      </c>
       <c r="U123" s="12">
         <v>66</v>
       </c>
@@ -6302,6 +6491,9 @@
         <f t="array" ref="S124">INDEX($I$6:$I$68, INT((ROWS(S$6:S124)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T124">
+        <v>3</v>
+      </c>
       <c r="U124" s="12">
         <v>61.18</v>
       </c>
@@ -6331,6 +6523,9 @@
         <f t="array" ref="S125">INDEX($I$6:$I$68, INT((ROWS(S$6:S125)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T125">
+        <v>3</v>
+      </c>
       <c r="U125" s="12">
         <v>65.709999999999994</v>
       </c>
@@ -6360,6 +6555,9 @@
         <f t="array" ref="S126">INDEX($I$6:$I$68, INT((ROWS(S$6:S126)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T126">
+        <v>1</v>
+      </c>
       <c r="U126" s="12">
         <v>90.22</v>
       </c>
@@ -6389,6 +6587,9 @@
         <f t="array" ref="S127">INDEX($I$6:$I$68, INT((ROWS(S$6:S127)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T127">
+        <v>1</v>
+      </c>
       <c r="U127" s="12">
         <v>81.08</v>
       </c>
@@ -6422,6 +6623,9 @@
         <f t="array" ref="S128">INDEX($I$6:$I$68, INT((ROWS(S$6:S128)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T128">
+        <v>1</v>
+      </c>
       <c r="U128" s="12">
         <v>74.010000000000005</v>
       </c>
@@ -6459,6 +6663,9 @@
         <f t="array" ref="S129">INDEX($I$6:$I$68, INT((ROWS(S$6:S129)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T129">
+        <v>1</v>
+      </c>
       <c r="U129" s="12">
         <v>72.37</v>
       </c>
@@ -6492,6 +6699,9 @@
         <f t="array" ref="S130">INDEX($I$6:$I$68, INT((ROWS(S$6:S130)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T130">
+        <v>1</v>
+      </c>
       <c r="U130" s="12">
         <v>89.44</v>
       </c>
@@ -6525,6 +6735,9 @@
         <f t="array" ref="S131">INDEX($I$6:$I$68, INT((ROWS(S$6:S131)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T131">
+        <v>2</v>
+      </c>
       <c r="U131" s="12">
         <v>65.7</v>
       </c>
@@ -6554,6 +6767,9 @@
         <f t="array" ref="S132">INDEX($I$6:$I$68, INT((ROWS(S$6:S132)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T132">
+        <v>2</v>
+      </c>
       <c r="U132" s="12">
         <v>60.51</v>
       </c>
@@ -6587,6 +6803,9 @@
         <f t="array" ref="S133">INDEX($I$6:$I$68, INT((ROWS(S$6:S133)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T133">
+        <v>2</v>
+      </c>
       <c r="U133" s="12">
         <v>71.819999999999993</v>
       </c>
@@ -6620,6 +6839,9 @@
         <f t="array" ref="S134">INDEX($I$6:$I$68, INT((ROWS(S$6:S134)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T134">
+        <v>2</v>
+      </c>
       <c r="U134" s="12">
         <v>61.53</v>
       </c>
@@ -6657,6 +6879,9 @@
         <f t="array" ref="S135">INDEX($I$6:$I$68, INT((ROWS(S$6:S135)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T135">
+        <v>2</v>
+      </c>
       <c r="U135" s="12">
         <v>63.02</v>
       </c>
@@ -6690,6 +6915,9 @@
         <f t="array" ref="S136">INDEX($I$6:$I$68, INT((ROWS(S$6:S136)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T136">
+        <v>3</v>
+      </c>
       <c r="U136" s="12">
         <v>57.89</v>
       </c>
@@ -6719,6 +6947,9 @@
         <f t="array" ref="S137">INDEX($I$6:$I$68, INT((ROWS(S$6:S137)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T137">
+        <v>3</v>
+      </c>
       <c r="U137" s="12">
         <v>49.75</v>
       </c>
@@ -6752,6 +6983,9 @@
         <f t="array" ref="S138">INDEX($I$6:$I$68, INT((ROWS(S$6:S138)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T138">
+        <v>3</v>
+      </c>
       <c r="U138" s="12">
         <v>53.04</v>
       </c>
@@ -6789,6 +7023,9 @@
         <f t="array" ref="S139">INDEX($I$6:$I$68, INT((ROWS(S$6:S139)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T139">
+        <v>3</v>
+      </c>
       <c r="U139" s="12">
         <v>45.62</v>
       </c>
@@ -6822,6 +7059,9 @@
         <f t="array" ref="S140">INDEX($I$6:$I$68, INT((ROWS(S$6:S140)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T140">
+        <v>3</v>
+      </c>
       <c r="U140" s="12">
         <v>46.48</v>
       </c>
@@ -6855,6 +7095,9 @@
         <f t="array" ref="S141">INDEX($I$6:$I$68, INT((ROWS(S$6:S141)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T141">
+        <v>1</v>
+      </c>
       <c r="U141" s="12">
         <v>99.46</v>
       </c>
@@ -6884,6 +7127,9 @@
         <f t="array" ref="S142">INDEX($I$6:$I$68, INT((ROWS(S$6:S142)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T142">
+        <v>1</v>
+      </c>
       <c r="U142" s="12">
         <v>68</v>
       </c>
@@ -6913,6 +7159,9 @@
         <f t="array" ref="S143">INDEX($I$6:$I$68, INT((ROWS(S$6:S143)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T143">
+        <v>1</v>
+      </c>
       <c r="U143" s="12">
         <v>76.959999999999994</v>
       </c>
@@ -6942,6 +7191,9 @@
         <f t="array" ref="S144">INDEX($I$6:$I$68, INT((ROWS(S$6:S144)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T144">
+        <v>1</v>
+      </c>
       <c r="U144" s="12">
         <v>70.72</v>
       </c>
@@ -6971,6 +7223,9 @@
         <f t="array" ref="S145">INDEX($I$6:$I$68, INT((ROWS(S$6:S145)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T145">
+        <v>1</v>
+      </c>
       <c r="U145" s="12">
         <v>87.25</v>
       </c>
@@ -7000,6 +7255,9 @@
         <f t="array" ref="S146">INDEX($I$6:$I$68, INT((ROWS(S$6:S146)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T146">
+        <v>2</v>
+      </c>
       <c r="U146" s="12">
         <v>93.01</v>
       </c>
@@ -7029,6 +7287,9 @@
         <f t="array" ref="S147">INDEX($I$6:$I$68, INT((ROWS(S$6:S147)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T147">
+        <v>2</v>
+      </c>
       <c r="U147" s="12">
         <v>110.65</v>
       </c>
@@ -7058,6 +7319,9 @@
         <f t="array" ref="S148">INDEX($I$6:$I$68, INT((ROWS(S$6:S148)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T148">
+        <v>2</v>
+      </c>
       <c r="U148" s="12">
         <v>93.11</v>
       </c>
@@ -7087,6 +7351,9 @@
         <f t="array" ref="S149">INDEX($I$6:$I$68, INT((ROWS(S$6:S149)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T149">
+        <v>2</v>
+      </c>
       <c r="U149" s="12">
         <v>99.13</v>
       </c>
@@ -7116,6 +7383,9 @@
         <f t="array" ref="S150">INDEX($I$6:$I$68, INT((ROWS(S$6:S150)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T150">
+        <v>2</v>
+      </c>
       <c r="U150" s="12">
         <v>87.89</v>
       </c>
@@ -7145,6 +7415,9 @@
         <f t="array" ref="S151">INDEX($I$6:$I$68, INT((ROWS(S$6:S151)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T151">
+        <v>3</v>
+      </c>
       <c r="U151" s="12">
         <v>76.010000000000005</v>
       </c>
@@ -7174,6 +7447,9 @@
         <f t="array" ref="S152">INDEX($I$6:$I$68, INT((ROWS(S$6:S152)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T152">
+        <v>3</v>
+      </c>
       <c r="U152" s="12">
         <v>111.12</v>
       </c>
@@ -7203,6 +7479,9 @@
         <f t="array" ref="S153">INDEX($I$6:$I$68, INT((ROWS(S$6:S153)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T153">
+        <v>3</v>
+      </c>
       <c r="U153" s="12">
         <v>87.73</v>
       </c>
@@ -7232,6 +7511,9 @@
         <f t="array" ref="S154">INDEX($I$6:$I$68, INT((ROWS(S$6:S154)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T154">
+        <v>3</v>
+      </c>
       <c r="U154" s="12">
         <v>73.52</v>
       </c>
@@ -7261,6 +7543,9 @@
         <f t="array" ref="S155">INDEX($I$6:$I$68, INT((ROWS(S$6:S155)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T155">
+        <v>3</v>
+      </c>
       <c r="U155" s="12">
         <v>94.78</v>
       </c>
@@ -7290,6 +7575,9 @@
         <f t="array" ref="S156">INDEX($I$6:$I$68, INT((ROWS(S$6:S156)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T156">
+        <v>1</v>
+      </c>
       <c r="U156" s="12">
         <v>91.19</v>
       </c>
@@ -7319,6 +7607,9 @@
         <f t="array" ref="S157">INDEX($I$6:$I$68, INT((ROWS(S$6:S157)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T157">
+        <v>1</v>
+      </c>
       <c r="U157" s="12">
         <v>88.86</v>
       </c>
@@ -7348,6 +7639,9 @@
         <f t="array" ref="S158">INDEX($I$6:$I$68, INT((ROWS(S$6:S158)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T158">
+        <v>1</v>
+      </c>
       <c r="U158" s="12">
         <v>91.21</v>
       </c>
@@ -7377,6 +7671,9 @@
         <f t="array" ref="S159">INDEX($I$6:$I$68, INT((ROWS(S$6:S159)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T159">
+        <v>1</v>
+      </c>
       <c r="U159" s="12">
         <v>86.01</v>
       </c>
@@ -7406,6 +7703,9 @@
         <f t="array" ref="S160">INDEX($I$6:$I$68, INT((ROWS(S$6:S160)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T160">
+        <v>1</v>
+      </c>
       <c r="U160" s="12">
         <v>72.650000000000006</v>
       </c>
@@ -7439,6 +7739,9 @@
         <f t="array" ref="S161">INDEX($I$6:$I$68, INT((ROWS(S$6:S161)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T161">
+        <v>2</v>
+      </c>
       <c r="U161" s="12">
         <v>84.74</v>
       </c>
@@ -7468,6 +7771,9 @@
         <f t="array" ref="S162">INDEX($I$6:$I$68, INT((ROWS(S$6:S162)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T162">
+        <v>2</v>
+      </c>
       <c r="U162" s="12">
         <v>67.510000000000005</v>
       </c>
@@ -7497,6 +7803,9 @@
         <f t="array" ref="S163">INDEX($I$6:$I$68, INT((ROWS(S$6:S163)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T163">
+        <v>2</v>
+      </c>
       <c r="U163" s="12">
         <v>68.64</v>
       </c>
@@ -7526,6 +7835,9 @@
         <f t="array" ref="S164">INDEX($I$6:$I$68, INT((ROWS(S$6:S164)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T164">
+        <v>2</v>
+      </c>
       <c r="U164" s="12">
         <v>75.62</v>
       </c>
@@ -7555,6 +7867,9 @@
         <f t="array" ref="S165">INDEX($I$6:$I$68, INT((ROWS(S$6:S165)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T165">
+        <v>2</v>
+      </c>
       <c r="U165" s="12">
         <v>73.27</v>
       </c>
@@ -7588,6 +7903,9 @@
         <f t="array" ref="S166">INDEX($I$6:$I$68, INT((ROWS(S$6:S166)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T166">
+        <v>3</v>
+      </c>
       <c r="U166" s="12">
         <v>58.74</v>
       </c>
@@ -7617,6 +7935,9 @@
         <f t="array" ref="S167">INDEX($I$6:$I$68, INT((ROWS(S$6:S167)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T167">
+        <v>3</v>
+      </c>
       <c r="U167" s="12">
         <v>64.459999999999994</v>
       </c>
@@ -7646,6 +7967,9 @@
         <f t="array" ref="S168">INDEX($I$6:$I$68, INT((ROWS(S$6:S168)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T168">
+        <v>3</v>
+      </c>
       <c r="U168" s="12">
         <v>59.31</v>
       </c>
@@ -7675,6 +7999,9 @@
         <f t="array" ref="S169">INDEX($I$6:$I$68, INT((ROWS(S$6:S169)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T169">
+        <v>3</v>
+      </c>
       <c r="U169" s="12">
         <v>61.3</v>
       </c>
@@ -7704,6 +8031,9 @@
         <f t="array" ref="S170">INDEX($I$6:$I$68, INT((ROWS(S$6:S170)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T170">
+        <v>3</v>
+      </c>
       <c r="U170" s="12">
         <v>61.91</v>
       </c>
@@ -7737,6 +8067,9 @@
         <f t="array" ref="S171">INDEX($I$6:$I$68, INT((ROWS(S$6:S171)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T171">
+        <v>1</v>
+      </c>
       <c r="U171" s="12">
         <v>70.78</v>
       </c>
@@ -7766,6 +8099,9 @@
         <f t="array" ref="S172">INDEX($I$6:$I$68, INT((ROWS(S$6:S172)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T172">
+        <v>1</v>
+      </c>
       <c r="U172" s="12">
         <v>65.680000000000007</v>
       </c>
@@ -7795,6 +8131,9 @@
         <f t="array" ref="S173">INDEX($I$6:$I$68, INT((ROWS(S$6:S173)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T173">
+        <v>1</v>
+      </c>
       <c r="U173" s="12">
         <v>66.3</v>
       </c>
@@ -7824,6 +8163,9 @@
         <f t="array" ref="S174">INDEX($I$6:$I$68, INT((ROWS(S$6:S174)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T174">
+        <v>1</v>
+      </c>
       <c r="U174" s="12">
         <v>72.59</v>
       </c>
@@ -7853,6 +8195,9 @@
         <f t="array" ref="S175">INDEX($I$6:$I$68, INT((ROWS(S$6:S175)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T175">
+        <v>1</v>
+      </c>
       <c r="U175" s="12">
         <v>62.11</v>
       </c>
@@ -7882,6 +8227,9 @@
         <f t="array" ref="S176">INDEX($I$6:$I$68, INT((ROWS(S$6:S176)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T176">
+        <v>2</v>
+      </c>
       <c r="U176" s="12">
         <v>54.88</v>
       </c>
@@ -7911,6 +8259,9 @@
         <f t="array" ref="S177">INDEX($I$6:$I$68, INT((ROWS(S$6:S177)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T177">
+        <v>2</v>
+      </c>
       <c r="U177" s="12">
         <v>47.98</v>
       </c>
@@ -7940,6 +8291,9 @@
         <f t="array" ref="S178">INDEX($I$6:$I$68, INT((ROWS(S$6:S178)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T178">
+        <v>2</v>
+      </c>
       <c r="U178" s="12">
         <v>49.79</v>
       </c>
@@ -7969,6 +8323,9 @@
         <f t="array" ref="S179">INDEX($I$6:$I$68, INT((ROWS(S$6:S179)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T179">
+        <v>2</v>
+      </c>
       <c r="U179" s="12">
         <v>53.31</v>
       </c>
@@ -7998,6 +8355,9 @@
         <f t="array" ref="S180">INDEX($I$6:$I$68, INT((ROWS(S$6:S180)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T180">
+        <v>2</v>
+      </c>
       <c r="U180" s="12">
         <v>47.59</v>
       </c>
@@ -8027,6 +8387,9 @@
         <f t="array" ref="S181">INDEX($I$6:$I$68, INT((ROWS(S$6:S181)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T181">
+        <v>3</v>
+      </c>
       <c r="U181" s="12">
         <v>72.45</v>
       </c>
@@ -8056,6 +8419,9 @@
         <f t="array" ref="S182">INDEX($I$6:$I$68, INT((ROWS(S$6:S182)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T182">
+        <v>3</v>
+      </c>
       <c r="U182" s="12">
         <v>78.7</v>
       </c>
@@ -8085,6 +8451,9 @@
         <f t="array" ref="S183">INDEX($I$6:$I$68, INT((ROWS(S$6:S183)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T183">
+        <v>3</v>
+      </c>
       <c r="U183" s="12">
         <v>66.87</v>
       </c>
@@ -8114,6 +8483,9 @@
         <f t="array" ref="S184">INDEX($I$6:$I$68, INT((ROWS(S$6:S184)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T184">
+        <v>3</v>
+      </c>
       <c r="U184" s="12">
         <v>81.459999999999994</v>
       </c>
@@ -8143,6 +8515,9 @@
         <f t="array" ref="S185">INDEX($I$6:$I$68, INT((ROWS(S$6:S185)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T185">
+        <v>3</v>
+      </c>
       <c r="U185" s="12">
         <v>64.77</v>
       </c>
@@ -8172,6 +8547,9 @@
         <f t="array" ref="S186">INDEX($I$6:$I$68, INT((ROWS(S$6:S186)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T186">
+        <v>1</v>
+      </c>
       <c r="U186" s="12">
         <v>82.2</v>
       </c>
@@ -8201,6 +8579,9 @@
         <f t="array" ref="S187">INDEX($I$6:$I$68, INT((ROWS(S$6:S187)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T187">
+        <v>1</v>
+      </c>
       <c r="U187" s="12">
         <v>76.709999999999994</v>
       </c>
@@ -8230,6 +8611,9 @@
         <f t="array" ref="S188">INDEX($I$6:$I$68, INT((ROWS(S$6:S188)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T188">
+        <v>1</v>
+      </c>
       <c r="U188" s="12">
         <v>76.2</v>
       </c>
@@ -8259,6 +8643,9 @@
         <f t="array" ref="S189">INDEX($I$6:$I$68, INT((ROWS(S$6:S189)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T189">
+        <v>1</v>
+      </c>
       <c r="U189" s="12">
         <v>80.680000000000007</v>
       </c>
@@ -8288,6 +8675,9 @@
         <f t="array" ref="S190">INDEX($I$6:$I$68, INT((ROWS(S$6:S190)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T190">
+        <v>1</v>
+      </c>
       <c r="U190" s="12">
         <v>73.239999999999995</v>
       </c>
@@ -8317,6 +8707,9 @@
         <f t="array" ref="S191">INDEX($I$6:$I$68, INT((ROWS(S$6:S191)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T191">
+        <v>2</v>
+      </c>
       <c r="U191" s="12">
         <v>88.99</v>
       </c>
@@ -8346,6 +8739,9 @@
         <f t="array" ref="S192">INDEX($I$6:$I$68, INT((ROWS(S$6:S192)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T192">
+        <v>2</v>
+      </c>
       <c r="U192" s="12">
         <v>74.099999999999994</v>
       </c>
@@ -8375,6 +8771,9 @@
         <f t="array" ref="S193">INDEX($I$6:$I$68, INT((ROWS(S$6:S193)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T193">
+        <v>2</v>
+      </c>
       <c r="U193" s="12">
         <v>85.46</v>
       </c>
@@ -8404,6 +8803,9 @@
         <f t="array" ref="S194">INDEX($I$6:$I$68, INT((ROWS(S$6:S194)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T194">
+        <v>2</v>
+      </c>
       <c r="U194" s="12">
         <v>83.88</v>
       </c>
@@ -8433,6 +8835,9 @@
         <f t="array" ref="S195">INDEX($I$6:$I$68, INT((ROWS(S$6:S195)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T195">
+        <v>2</v>
+      </c>
       <c r="U195" s="12">
         <v>70.739999999999995</v>
       </c>
@@ -8462,6 +8867,9 @@
         <f t="array" ref="S196">INDEX($I$6:$I$68, INT((ROWS(S$6:S196)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T196">
+        <v>3</v>
+      </c>
       <c r="U196" s="12">
         <v>70.84</v>
       </c>
@@ -8491,6 +8899,9 @@
         <f t="array" ref="S197">INDEX($I$6:$I$68, INT((ROWS(S$6:S197)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T197">
+        <v>3</v>
+      </c>
       <c r="U197" s="12">
         <v>57.39</v>
       </c>
@@ -8520,6 +8931,9 @@
         <f t="array" ref="S198">INDEX($I$6:$I$68, INT((ROWS(S$6:S198)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T198">
+        <v>3</v>
+      </c>
       <c r="U198" s="12">
         <v>56.09</v>
       </c>
@@ -8549,6 +8963,9 @@
         <f t="array" ref="S199">INDEX($I$6:$I$68, INT((ROWS(S$6:S199)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T199">
+        <v>3</v>
+      </c>
       <c r="U199" s="12">
         <v>52.68</v>
       </c>
@@ -8578,6 +8995,9 @@
         <f t="array" ref="S200">INDEX($I$6:$I$68, INT((ROWS(S$6:S200)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T200">
+        <v>3</v>
+      </c>
       <c r="U200" s="12">
         <v>51.96</v>
       </c>
@@ -8607,6 +9027,9 @@
         <f t="array" ref="S201">INDEX($I$6:$I$68, INT((ROWS(S$6:S201)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T201">
+        <v>1</v>
+      </c>
       <c r="U201" s="12">
         <v>75.06</v>
       </c>
@@ -8636,6 +9059,9 @@
         <f t="array" ref="S202">INDEX($I$6:$I$68, INT((ROWS(S$6:S202)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T202">
+        <v>1</v>
+      </c>
       <c r="U202" s="12">
         <v>76.69</v>
       </c>
@@ -8665,6 +9091,9 @@
         <f t="array" ref="S203">INDEX($I$6:$I$68, INT((ROWS(S$6:S203)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T203">
+        <v>1</v>
+      </c>
       <c r="U203" s="12">
         <v>68.03</v>
       </c>
@@ -8694,6 +9123,9 @@
         <f t="array" ref="S204">INDEX($I$6:$I$68, INT((ROWS(S$6:S204)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T204">
+        <v>1</v>
+      </c>
       <c r="U204" s="12">
         <v>65.16</v>
       </c>
@@ -8723,6 +9155,9 @@
         <f t="array" ref="S205">INDEX($I$6:$I$68, INT((ROWS(S$6:S205)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T205">
+        <v>1</v>
+      </c>
       <c r="U205" s="12">
         <v>73.349999999999994</v>
       </c>
@@ -8752,6 +9187,9 @@
         <f t="array" ref="S206">INDEX($I$6:$I$68, INT((ROWS(S$6:S206)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T206">
+        <v>2</v>
+      </c>
       <c r="U206" s="12">
         <v>50.14</v>
       </c>
@@ -8781,6 +9219,9 @@
         <f t="array" ref="S207">INDEX($I$6:$I$68, INT((ROWS(S$6:S207)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T207">
+        <v>2</v>
+      </c>
       <c r="U207" s="12">
         <v>49.65</v>
       </c>
@@ -8810,6 +9251,9 @@
         <f t="array" ref="S208">INDEX($I$6:$I$68, INT((ROWS(S$6:S208)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T208">
+        <v>2</v>
+      </c>
       <c r="U208" s="12">
         <v>48.16</v>
       </c>
@@ -8839,6 +9283,9 @@
         <f t="array" ref="S209">INDEX($I$6:$I$68, INT((ROWS(S$6:S209)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T209">
+        <v>2</v>
+      </c>
       <c r="U209" s="12">
         <v>56.64</v>
       </c>
@@ -8868,6 +9315,9 @@
         <f t="array" ref="S210">INDEX($I$6:$I$68, INT((ROWS(S$6:S210)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T210">
+        <v>2</v>
+      </c>
       <c r="U210" s="12">
         <v>53.8</v>
       </c>
@@ -8897,6 +9347,9 @@
         <f t="array" ref="S211">INDEX($I$6:$I$68, INT((ROWS(S$6:S211)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T211">
+        <v>3</v>
+      </c>
       <c r="U211" s="12">
         <v>93.1</v>
       </c>
@@ -8926,6 +9379,9 @@
         <f t="array" ref="S212">INDEX($I$6:$I$68, INT((ROWS(S$6:S212)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T212">
+        <v>3</v>
+      </c>
       <c r="U212" s="12">
         <v>62.21</v>
       </c>
@@ -8955,6 +9411,9 @@
         <f t="array" ref="S213">INDEX($I$6:$I$68, INT((ROWS(S$6:S213)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T213">
+        <v>3</v>
+      </c>
       <c r="U213" s="12">
         <v>62.55</v>
       </c>
@@ -8984,6 +9443,9 @@
         <f t="array" ref="S214">INDEX($I$6:$I$68, INT((ROWS(S$6:S214)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T214">
+        <v>3</v>
+      </c>
       <c r="U214" s="12">
         <v>64.010000000000005</v>
       </c>
@@ -9013,6 +9475,9 @@
         <f t="array" ref="S215">INDEX($I$6:$I$68, INT((ROWS(S$6:S215)-1)/5)+1)</f>
         <v>2</v>
       </c>
+      <c r="T215">
+        <v>3</v>
+      </c>
       <c r="U215" s="12">
         <v>71.38</v>
       </c>
@@ -9042,6 +9507,9 @@
         <f t="array" ref="S216">INDEX($I$6:$I$68, INT((ROWS(S$6:S216)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T216">
+        <v>1</v>
+      </c>
       <c r="U216" s="12">
         <v>50.74</v>
       </c>
@@ -9071,6 +9539,9 @@
         <f t="array" ref="S217">INDEX($I$6:$I$68, INT((ROWS(S$6:S217)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T217">
+        <v>1</v>
+      </c>
       <c r="U217" s="12">
         <v>50.82</v>
       </c>
@@ -9100,6 +9571,9 @@
         <f t="array" ref="S218">INDEX($I$6:$I$68, INT((ROWS(S$6:S218)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T218">
+        <v>1</v>
+      </c>
       <c r="U218" s="12">
         <v>49.66</v>
       </c>
@@ -9129,6 +9603,9 @@
         <f t="array" ref="S219">INDEX($I$6:$I$68, INT((ROWS(S$6:S219)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T219">
+        <v>1</v>
+      </c>
       <c r="U219" s="12">
         <v>49.87</v>
       </c>
@@ -9158,6 +9635,9 @@
         <f t="array" ref="S220">INDEX($I$6:$I$68, INT((ROWS(S$6:S220)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T220">
+        <v>1</v>
+      </c>
       <c r="U220" s="12">
         <v>45.18</v>
       </c>
@@ -9187,6 +9667,9 @@
         <f t="array" ref="S221">INDEX($I$6:$I$68, INT((ROWS(S$6:S221)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T221">
+        <v>2</v>
+      </c>
       <c r="U221" s="12">
         <v>68.05</v>
       </c>
@@ -9216,6 +9699,9 @@
         <f t="array" ref="S222">INDEX($I$6:$I$68, INT((ROWS(S$6:S222)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T222">
+        <v>2</v>
+      </c>
       <c r="U222" s="12">
         <v>60.38</v>
       </c>
@@ -9245,6 +9731,9 @@
         <f t="array" ref="S223">INDEX($I$6:$I$68, INT((ROWS(S$6:S223)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T223">
+        <v>2</v>
+      </c>
       <c r="U223" s="12">
         <v>59.31</v>
       </c>
@@ -9274,6 +9763,9 @@
         <f t="array" ref="S224">INDEX($I$6:$I$68, INT((ROWS(S$6:S224)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T224">
+        <v>2</v>
+      </c>
       <c r="U224" s="12">
         <v>65.849999999999994</v>
       </c>
@@ -9303,6 +9795,9 @@
         <f t="array" ref="S225">INDEX($I$6:$I$68, INT((ROWS(S$6:S225)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T225">
+        <v>2</v>
+      </c>
       <c r="U225" s="12">
         <v>62.58</v>
       </c>
@@ -9332,6 +9827,9 @@
         <f t="array" ref="S226">INDEX($I$6:$I$68, INT((ROWS(S$6:S226)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T226">
+        <v>3</v>
+      </c>
       <c r="U226" s="12">
         <v>74.59</v>
       </c>
@@ -9361,6 +9859,9 @@
         <f t="array" ref="S227">INDEX($I$6:$I$68, INT((ROWS(S$6:S227)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T227">
+        <v>3</v>
+      </c>
       <c r="U227" s="12">
         <v>62.07</v>
       </c>
@@ -9390,6 +9891,9 @@
         <f t="array" ref="S228">INDEX($I$6:$I$68, INT((ROWS(S$6:S228)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T228">
+        <v>3</v>
+      </c>
       <c r="U228" s="12">
         <v>60.93</v>
       </c>
@@ -9419,6 +9923,9 @@
         <f t="array" ref="S229">INDEX($I$6:$I$68, INT((ROWS(S$6:S229)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T229">
+        <v>3</v>
+      </c>
       <c r="U229" s="12">
         <v>61.43</v>
       </c>
@@ -9448,6 +9955,9 @@
         <f t="array" ref="S230">INDEX($I$6:$I$68, INT((ROWS(S$6:S230)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T230">
+        <v>3</v>
+      </c>
       <c r="U230" s="12">
         <v>64.3</v>
       </c>
@@ -9477,6 +9987,9 @@
         <f t="array" ref="S231">INDEX($I$6:$I$68, INT((ROWS(S$6:S231)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T231">
+        <v>1</v>
+      </c>
       <c r="U231" s="12">
         <v>69.44</v>
       </c>
@@ -9506,6 +10019,9 @@
         <f t="array" ref="S232">INDEX($I$6:$I$68, INT((ROWS(S$6:S232)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T232">
+        <v>1</v>
+      </c>
       <c r="U232" s="12">
         <v>59.19</v>
       </c>
@@ -9535,6 +10051,9 @@
         <f t="array" ref="S233">INDEX($I$6:$I$68, INT((ROWS(S$6:S233)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T233">
+        <v>1</v>
+      </c>
       <c r="U233" s="12">
         <v>60.08</v>
       </c>
@@ -9564,6 +10083,9 @@
         <f t="array" ref="S234">INDEX($I$6:$I$68, INT((ROWS(S$6:S234)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T234">
+        <v>1</v>
+      </c>
       <c r="U234" s="12">
         <v>59.64</v>
       </c>
@@ -9593,6 +10115,9 @@
         <f t="array" ref="S235">INDEX($I$6:$I$68, INT((ROWS(S$6:S235)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T235">
+        <v>1</v>
+      </c>
       <c r="U235" s="12">
         <v>60.08</v>
       </c>
@@ -9622,6 +10147,9 @@
         <f t="array" ref="S236">INDEX($I$6:$I$68, INT((ROWS(S$6:S236)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T236">
+        <v>2</v>
+      </c>
       <c r="U236" s="12">
         <v>47.79</v>
       </c>
@@ -9651,6 +10179,9 @@
         <f t="array" ref="S237">INDEX($I$6:$I$68, INT((ROWS(S$6:S237)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T237">
+        <v>2</v>
+      </c>
       <c r="U237" s="12">
         <v>43.56</v>
       </c>
@@ -9680,6 +10211,9 @@
         <f t="array" ref="S238">INDEX($I$6:$I$68, INT((ROWS(S$6:S238)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T238">
+        <v>2</v>
+      </c>
       <c r="U238" s="12">
         <v>44.25</v>
       </c>
@@ -9709,6 +10243,9 @@
         <f t="array" ref="S239">INDEX($I$6:$I$68, INT((ROWS(S$6:S239)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T239">
+        <v>2</v>
+      </c>
       <c r="U239" s="12">
         <v>43.61</v>
       </c>
@@ -9738,6 +10275,9 @@
         <f t="array" ref="S240">INDEX($I$6:$I$68, INT((ROWS(S$6:S240)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T240">
+        <v>2</v>
+      </c>
       <c r="U240" s="12">
         <v>44.65</v>
       </c>
@@ -9767,7 +10307,12 @@
         <f t="array" ref="S241">INDEX($I$6:$I$68, INT((ROWS(S$6:S241)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U241" s="12"/>
+      <c r="T241">
+        <v>3</v>
+      </c>
+      <c r="U241" s="12">
+        <v>64.61</v>
+      </c>
     </row>
     <row r="242" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N242" s="2" t="str">
@@ -9794,7 +10339,12 @@
         <f t="array" ref="S242">INDEX($I$6:$I$68, INT((ROWS(S$6:S242)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U242" s="12"/>
+      <c r="T242">
+        <v>3</v>
+      </c>
+      <c r="U242" s="12">
+        <v>56.59</v>
+      </c>
     </row>
     <row r="243" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N243" s="2" t="str">
@@ -9821,7 +10371,12 @@
         <f t="array" ref="S243">INDEX($I$6:$I$68, INT((ROWS(S$6:S243)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U243" s="12"/>
+      <c r="T243">
+        <v>3</v>
+      </c>
+      <c r="U243" s="12">
+        <v>56.99</v>
+      </c>
     </row>
     <row r="244" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N244" s="2" t="str">
@@ -9848,7 +10403,12 @@
         <f t="array" ref="S244">INDEX($I$6:$I$68, INT((ROWS(S$6:S244)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U244" s="12"/>
+      <c r="T244">
+        <v>3</v>
+      </c>
+      <c r="U244" s="12">
+        <v>58.66</v>
+      </c>
     </row>
     <row r="245" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N245" s="2" t="str">
@@ -9875,7 +10435,12 @@
         <f t="array" ref="S245">INDEX($I$6:$I$68, INT((ROWS(S$6:S245)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U245" s="12"/>
+      <c r="T245">
+        <v>3</v>
+      </c>
+      <c r="U245" s="12">
+        <v>56.99</v>
+      </c>
     </row>
     <row r="246" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N246" s="2" t="str">
@@ -9902,6 +10467,9 @@
         <f t="array" ref="S246">INDEX($I$6:$I$68, INT((ROWS(S$6:S246)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T246">
+        <v>1</v>
+      </c>
       <c r="U246" s="12">
         <v>49.82</v>
       </c>
@@ -9931,6 +10499,9 @@
         <f t="array" ref="S247">INDEX($I$6:$I$68, INT((ROWS(S$6:S247)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T247">
+        <v>1</v>
+      </c>
       <c r="U247" s="12">
         <v>46.03</v>
       </c>
@@ -9960,6 +10531,9 @@
         <f t="array" ref="S248">INDEX($I$6:$I$68, INT((ROWS(S$6:S248)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T248">
+        <v>1</v>
+      </c>
       <c r="U248" s="12">
         <v>42.73</v>
       </c>
@@ -9989,6 +10563,9 @@
         <f t="array" ref="S249">INDEX($I$6:$I$68, INT((ROWS(S$6:S249)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T249">
+        <v>1</v>
+      </c>
       <c r="U249" s="12">
         <v>44.59</v>
       </c>
@@ -10018,6 +10595,9 @@
         <f t="array" ref="S250">INDEX($I$6:$I$68, INT((ROWS(S$6:S250)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T250">
+        <v>1</v>
+      </c>
       <c r="U250" s="12">
         <v>43.89</v>
       </c>
@@ -10047,6 +10627,9 @@
         <f t="array" ref="S251">INDEX($I$6:$I$68, INT((ROWS(S$6:S251)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T251">
+        <v>2</v>
+      </c>
       <c r="U251" s="12">
         <v>60.04</v>
       </c>
@@ -10076,6 +10659,9 @@
         <f t="array" ref="S252">INDEX($I$6:$I$68, INT((ROWS(S$6:S252)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T252">
+        <v>2</v>
+      </c>
       <c r="U252" s="12">
         <v>55.78</v>
       </c>
@@ -10105,6 +10691,9 @@
         <f t="array" ref="S253">INDEX($I$6:$I$68, INT((ROWS(S$6:S253)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T253">
+        <v>2</v>
+      </c>
       <c r="U253" s="12">
         <v>65</v>
       </c>
@@ -10134,6 +10723,9 @@
         <f t="array" ref="S254">INDEX($I$6:$I$68, INT((ROWS(S$6:S254)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T254">
+        <v>2</v>
+      </c>
       <c r="U254" s="12">
         <v>55.56</v>
       </c>
@@ -10163,6 +10755,9 @@
         <f t="array" ref="S255">INDEX($I$6:$I$68, INT((ROWS(S$6:S255)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T255">
+        <v>2</v>
+      </c>
       <c r="U255" s="12">
         <v>54.2</v>
       </c>
@@ -10192,11 +10787,14 @@
         <f t="array" ref="S256">INDEX($I$6:$I$68, INT((ROWS(S$6:S256)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T256">
+        <v>3</v>
+      </c>
       <c r="U256" s="12">
         <v>60.52</v>
       </c>
     </row>
-    <row r="257" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="257" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N257" s="2" t="str">
         <f t="shared" si="8"/>
         <v>IA ID16</v>
@@ -10221,11 +10819,14 @@
         <f t="array" ref="S257">INDEX($I$6:$I$68, INT((ROWS(S$6:S257)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T257">
+        <v>3</v>
+      </c>
       <c r="U257" s="12">
         <v>56.38</v>
       </c>
     </row>
-    <row r="258" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="258" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N258" s="2" t="str">
         <f t="shared" si="8"/>
         <v>IA ID16</v>
@@ -10250,11 +10851,14 @@
         <f t="array" ref="S258">INDEX($I$6:$I$68, INT((ROWS(S$6:S258)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T258">
+        <v>3</v>
+      </c>
       <c r="U258" s="12">
         <v>56.54</v>
       </c>
     </row>
-    <row r="259" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="259" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N259" s="2" t="str">
         <f t="shared" si="8"/>
         <v>IA ID16</v>
@@ -10279,11 +10883,14 @@
         <f t="array" ref="S259">INDEX($I$6:$I$68, INT((ROWS(S$6:S259)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T259">
+        <v>3</v>
+      </c>
       <c r="U259" s="12">
         <v>55.03</v>
       </c>
     </row>
-    <row r="260" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="260" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N260" s="2" t="str">
         <f t="shared" si="8"/>
         <v>IA ID16</v>
@@ -10308,11 +10915,14 @@
         <f t="array" ref="S260">INDEX($I$6:$I$68, INT((ROWS(S$6:S260)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T260">
+        <v>3</v>
+      </c>
       <c r="U260" s="12">
         <v>56.02</v>
       </c>
     </row>
-    <row r="261" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="261" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N261" s="2" t="str">
         <f t="shared" si="8"/>
         <v>MaL ID19</v>
@@ -10337,14 +10947,14 @@
         <f t="array" ref="S261">INDEX($I$6:$I$68, INT((ROWS(S$6:S261)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T261">
+        <v>1</v>
+      </c>
       <c r="U261" s="12">
         <v>70</v>
       </c>
-      <c r="X261" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="262" spans="14:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="262" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N262" s="2" t="str">
         <f t="shared" si="8"/>
         <v>MaL ID19</v>
@@ -10369,14 +10979,14 @@
         <f t="array" ref="S262">INDEX($I$6:$I$68, INT((ROWS(S$6:S262)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T262">
+        <v>1</v>
+      </c>
       <c r="U262" s="12">
         <v>70</v>
       </c>
-      <c r="X262" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="263" spans="14:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="263" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N263" s="2" t="str">
         <f t="shared" ref="N263:N320" si="9">INDEX($B$6:$B$26, MATCH(O263, $A$6:$A$26, 0))</f>
         <v>MaL ID19</v>
@@ -10401,11 +11011,14 @@
         <f t="array" ref="S263">INDEX($I$6:$I$68, INT((ROWS(S$6:S263)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T263">
+        <v>1</v>
+      </c>
       <c r="U263" s="12">
         <v>74.95</v>
       </c>
     </row>
-    <row r="264" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="264" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N264" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10430,11 +11043,14 @@
         <f t="array" ref="S264">INDEX($I$6:$I$68, INT((ROWS(S$6:S264)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T264">
+        <v>1</v>
+      </c>
       <c r="U264" s="12">
         <v>63.85</v>
       </c>
     </row>
-    <row r="265" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="265" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N265" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10459,11 +11075,14 @@
         <f t="array" ref="S265">INDEX($I$6:$I$68, INT((ROWS(S$6:S265)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T265">
+        <v>1</v>
+      </c>
       <c r="U265" s="12">
         <v>64.849999999999994</v>
       </c>
     </row>
-    <row r="266" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="266" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N266" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10488,11 +11107,14 @@
         <f t="array" ref="S266">INDEX($I$6:$I$68, INT((ROWS(S$6:S266)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T266">
+        <v>2</v>
+      </c>
       <c r="U266" s="12">
         <v>76.91</v>
       </c>
     </row>
-    <row r="267" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="267" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N267" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10517,11 +11139,14 @@
         <f t="array" ref="S267">INDEX($I$6:$I$68, INT((ROWS(S$6:S267)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T267">
+        <v>2</v>
+      </c>
       <c r="U267" s="12">
         <v>64.11</v>
       </c>
     </row>
-    <row r="268" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="268" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N268" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10546,11 +11171,14 @@
         <f t="array" ref="S268">INDEX($I$6:$I$68, INT((ROWS(S$6:S268)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T268">
+        <v>2</v>
+      </c>
       <c r="U268" s="12">
         <v>68.040000000000006</v>
       </c>
     </row>
-    <row r="269" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="269" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N269" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10575,11 +11203,14 @@
         <f t="array" ref="S269">INDEX($I$6:$I$68, INT((ROWS(S$6:S269)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T269">
+        <v>2</v>
+      </c>
       <c r="U269" s="12">
         <v>64.88</v>
       </c>
     </row>
-    <row r="270" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="270" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N270" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10604,11 +11235,14 @@
         <f t="array" ref="S270">INDEX($I$6:$I$68, INT((ROWS(S$6:S270)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T270">
+        <v>2</v>
+      </c>
       <c r="U270" s="12">
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="271" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="271" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N271" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10633,11 +11267,14 @@
         <f t="array" ref="S271">INDEX($I$6:$I$68, INT((ROWS(S$6:S271)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T271">
+        <v>3</v>
+      </c>
       <c r="U271" s="12">
         <v>51.76</v>
       </c>
     </row>
-    <row r="272" spans="14:24" x14ac:dyDescent="0.25">
+    <row r="272" spans="14:21" x14ac:dyDescent="0.25">
       <c r="N272" s="2" t="str">
         <f t="shared" si="9"/>
         <v>MaL ID19</v>
@@ -10660,6 +11297,9 @@
       </c>
       <c r="S272" cm="1">
         <f t="array" ref="S272">INDEX($I$6:$I$68, INT((ROWS(S$6:S272)-1)/5)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="T272">
         <v>3</v>
       </c>
       <c r="U272" s="12">
@@ -10691,6 +11331,9 @@
         <f t="array" ref="S273">INDEX($I$6:$I$68, INT((ROWS(S$6:S273)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T273">
+        <v>3</v>
+      </c>
       <c r="U273" s="12">
         <v>48.12</v>
       </c>
@@ -10720,6 +11363,9 @@
         <f t="array" ref="S274">INDEX($I$6:$I$68, INT((ROWS(S$6:S274)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T274">
+        <v>3</v>
+      </c>
       <c r="U274" s="12">
         <v>47.78</v>
       </c>
@@ -10749,6 +11395,9 @@
         <f t="array" ref="S275">INDEX($I$6:$I$68, INT((ROWS(S$6:S275)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T275">
+        <v>3</v>
+      </c>
       <c r="U275" s="12">
         <v>45.45</v>
       </c>
@@ -10778,6 +11427,9 @@
         <f t="array" ref="S276">INDEX($I$6:$I$68, INT((ROWS(S$6:S276)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T276">
+        <v>1</v>
+      </c>
       <c r="U276" s="12">
         <v>64</v>
       </c>
@@ -10807,6 +11459,9 @@
         <f t="array" ref="S277">INDEX($I$6:$I$68, INT((ROWS(S$6:S277)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T277">
+        <v>1</v>
+      </c>
       <c r="U277" s="12">
         <v>51.63</v>
       </c>
@@ -10836,6 +11491,9 @@
         <f t="array" ref="S278">INDEX($I$6:$I$68, INT((ROWS(S$6:S278)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T278">
+        <v>1</v>
+      </c>
       <c r="U278" s="12">
         <v>54.36</v>
       </c>
@@ -10865,6 +11523,9 @@
         <f t="array" ref="S279">INDEX($I$6:$I$68, INT((ROWS(S$6:S279)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T279">
+        <v>1</v>
+      </c>
       <c r="U279" s="12">
         <v>52.93</v>
       </c>
@@ -10894,6 +11555,9 @@
         <f t="array" ref="S280">INDEX($I$6:$I$68, INT((ROWS(S$6:S280)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T280">
+        <v>1</v>
+      </c>
       <c r="U280" s="12">
         <v>51.12</v>
       </c>
@@ -10923,6 +11587,9 @@
         <f t="array" ref="S281">INDEX($I$6:$I$68, INT((ROWS(S$6:S281)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T281">
+        <v>2</v>
+      </c>
       <c r="U281" s="12">
         <v>85.88</v>
       </c>
@@ -10952,6 +11619,9 @@
         <f t="array" ref="S282">INDEX($I$6:$I$68, INT((ROWS(S$6:S282)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T282">
+        <v>2</v>
+      </c>
       <c r="U282" s="12">
         <v>70.98</v>
       </c>
@@ -10981,6 +11651,9 @@
         <f t="array" ref="S283">INDEX($I$6:$I$68, INT((ROWS(S$6:S283)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T283">
+        <v>2</v>
+      </c>
       <c r="U283" s="12">
         <v>71.72</v>
       </c>
@@ -11010,6 +11683,9 @@
         <f t="array" ref="S284">INDEX($I$6:$I$68, INT((ROWS(S$6:S284)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T284">
+        <v>2</v>
+      </c>
       <c r="U284" s="12">
         <v>72.09</v>
       </c>
@@ -11039,6 +11715,9 @@
         <f t="array" ref="S285">INDEX($I$6:$I$68, INT((ROWS(S$6:S285)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T285">
+        <v>2</v>
+      </c>
       <c r="U285" s="12">
         <v>71.819999999999993</v>
       </c>
@@ -11068,6 +11747,9 @@
         <f t="array" ref="S286">INDEX($I$6:$I$68, INT((ROWS(S$6:S286)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T286">
+        <v>3</v>
+      </c>
       <c r="U286" s="12">
         <v>72.040000000000006</v>
       </c>
@@ -11097,6 +11779,9 @@
         <f t="array" ref="S287">INDEX($I$6:$I$68, INT((ROWS(S$6:S287)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T287">
+        <v>3</v>
+      </c>
       <c r="U287" s="12">
         <v>68.48</v>
       </c>
@@ -11126,6 +11811,9 @@
         <f t="array" ref="S288">INDEX($I$6:$I$68, INT((ROWS(S$6:S288)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T288">
+        <v>3</v>
+      </c>
       <c r="U288" s="12">
         <v>66.209999999999994</v>
       </c>
@@ -11155,6 +11843,9 @@
         <f t="array" ref="S289">INDEX($I$6:$I$68, INT((ROWS(S$6:S289)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T289">
+        <v>3</v>
+      </c>
       <c r="U289" s="12">
         <v>66.42</v>
       </c>
@@ -11184,6 +11875,9 @@
         <f t="array" ref="S290">INDEX($I$6:$I$68, INT((ROWS(S$6:S290)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T290">
+        <v>3</v>
+      </c>
       <c r="U290" s="12">
         <v>67.44</v>
       </c>
@@ -11213,6 +11907,9 @@
         <f t="array" ref="S291">INDEX($I$6:$I$68, INT((ROWS(S$6:S291)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T291">
+        <v>1</v>
+      </c>
       <c r="U291" s="12">
         <v>62.25</v>
       </c>
@@ -11242,6 +11939,9 @@
         <f t="array" ref="S292">INDEX($I$6:$I$68, INT((ROWS(S$6:S292)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T292">
+        <v>1</v>
+      </c>
       <c r="U292" s="12">
         <v>59.29</v>
       </c>
@@ -11271,6 +11971,9 @@
         <f t="array" ref="S293">INDEX($I$6:$I$68, INT((ROWS(S$6:S293)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T293">
+        <v>1</v>
+      </c>
       <c r="U293" s="12">
         <v>59.1</v>
       </c>
@@ -11300,6 +12003,9 @@
         <f t="array" ref="S294">INDEX($I$6:$I$68, INT((ROWS(S$6:S294)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T294">
+        <v>1</v>
+      </c>
       <c r="U294" s="12">
         <v>58.8</v>
       </c>
@@ -11329,6 +12035,9 @@
         <f t="array" ref="S295">INDEX($I$6:$I$68, INT((ROWS(S$6:S295)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T295">
+        <v>1</v>
+      </c>
       <c r="U295" s="12">
         <v>58.69</v>
       </c>
@@ -11358,6 +12067,9 @@
         <f t="array" ref="S296">INDEX($I$6:$I$68, INT((ROWS(S$6:S296)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T296">
+        <v>2</v>
+      </c>
       <c r="U296" s="12">
         <v>61.12</v>
       </c>
@@ -11387,6 +12099,9 @@
         <f t="array" ref="S297">INDEX($I$6:$I$68, INT((ROWS(S$6:S297)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T297">
+        <v>2</v>
+      </c>
       <c r="U297" s="12">
         <v>59.87</v>
       </c>
@@ -11416,6 +12131,9 @@
         <f t="array" ref="S298">INDEX($I$6:$I$68, INT((ROWS(S$6:S298)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T298">
+        <v>2</v>
+      </c>
       <c r="U298" s="12">
         <v>57.7</v>
       </c>
@@ -11445,6 +12163,9 @@
         <f t="array" ref="S299">INDEX($I$6:$I$68, INT((ROWS(S$6:S299)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T299">
+        <v>2</v>
+      </c>
       <c r="U299" s="12">
         <v>58.65</v>
       </c>
@@ -11474,6 +12195,9 @@
         <f t="array" ref="S300">INDEX($I$6:$I$68, INT((ROWS(S$6:S300)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T300">
+        <v>2</v>
+      </c>
       <c r="U300" s="12">
         <v>57.7</v>
       </c>
@@ -11503,6 +12227,9 @@
         <f t="array" ref="S301">INDEX($I$6:$I$68, INT((ROWS(S$6:S301)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T301">
+        <v>3</v>
+      </c>
       <c r="U301" s="12">
         <v>46.18</v>
       </c>
@@ -11532,6 +12259,9 @@
         <f t="array" ref="S302">INDEX($I$6:$I$68, INT((ROWS(S$6:S302)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T302">
+        <v>3</v>
+      </c>
       <c r="U302" s="12">
         <v>42.67</v>
       </c>
@@ -11561,6 +12291,9 @@
         <f t="array" ref="S303">INDEX($I$6:$I$68, INT((ROWS(S$6:S303)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T303">
+        <v>3</v>
+      </c>
       <c r="U303" s="12">
         <v>43.4</v>
       </c>
@@ -11590,11 +12323,14 @@
         <f t="array" ref="S304">INDEX($I$6:$I$68, INT((ROWS(S$6:S304)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T304">
+        <v>3</v>
+      </c>
       <c r="U304" s="12">
         <v>42.46</v>
       </c>
     </row>
-    <row r="305" spans="14:21" x14ac:dyDescent="0.25">
+    <row r="305" spans="14:24" x14ac:dyDescent="0.25">
       <c r="N305" s="2" t="str">
         <f t="shared" si="9"/>
         <v>FW ID22</v>
@@ -11619,14 +12355,17 @@
         <f t="array" ref="S305">INDEX($I$6:$I$68, INT((ROWS(S$6:S305)-1)/5)+1)</f>
         <v>3</v>
       </c>
+      <c r="T305">
+        <v>3</v>
+      </c>
       <c r="U305" s="12">
         <v>43.76</v>
       </c>
     </row>
-    <row r="306" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N306" s="2">
+    <row r="306" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N306" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O306" cm="1">
         <f t="array" ref="O306">INDEX($F$6:$F$68, INT((ROWS(O$6:O306)-1)/5)+1)</f>
@@ -11648,12 +12387,17 @@
         <f t="array" ref="S306">INDEX($I$6:$I$68, INT((ROWS(S$6:S306)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U306" s="12"/>
-    </row>
-    <row r="307" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N307" s="2">
+      <c r="T306">
+        <v>1</v>
+      </c>
+      <c r="U306" s="12">
+        <v>82.13</v>
+      </c>
+    </row>
+    <row r="307" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N307" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O307" cm="1">
         <f t="array" ref="O307">INDEX($F$6:$F$68, INT((ROWS(O$6:O307)-1)/5)+1)</f>
@@ -11675,12 +12419,17 @@
         <f t="array" ref="S307">INDEX($I$6:$I$68, INT((ROWS(S$6:S307)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U307" s="12"/>
-    </row>
-    <row r="308" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N308" s="2">
+      <c r="T307">
+        <v>1</v>
+      </c>
+      <c r="U307" s="12">
+        <v>55.91</v>
+      </c>
+    </row>
+    <row r="308" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N308" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O308" cm="1">
         <f t="array" ref="O308">INDEX($F$6:$F$68, INT((ROWS(O$6:O308)-1)/5)+1)</f>
@@ -11702,12 +12451,17 @@
         <f t="array" ref="S308">INDEX($I$6:$I$68, INT((ROWS(S$6:S308)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U308" s="12"/>
-    </row>
-    <row r="309" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N309" s="2">
+      <c r="T308">
+        <v>1</v>
+      </c>
+      <c r="U308" s="12">
+        <v>54.77</v>
+      </c>
+    </row>
+    <row r="309" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N309" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O309" cm="1">
         <f t="array" ref="O309">INDEX($F$6:$F$68, INT((ROWS(O$6:O309)-1)/5)+1)</f>
@@ -11729,12 +12483,20 @@
         <f t="array" ref="S309">INDEX($I$6:$I$68, INT((ROWS(S$6:S309)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U309" s="12"/>
-    </row>
-    <row r="310" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N310" s="2">
+      <c r="T309">
+        <v>1</v>
+      </c>
+      <c r="U309" s="12">
+        <v>60.95</v>
+      </c>
+      <c r="X309" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="310" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N310" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O310" cm="1">
         <f t="array" ref="O310">INDEX($F$6:$F$68, INT((ROWS(O$6:O310)-1)/5)+1)</f>
@@ -11756,12 +12518,17 @@
         <f t="array" ref="S310">INDEX($I$6:$I$68, INT((ROWS(S$6:S310)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U310" s="12"/>
-    </row>
-    <row r="311" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N311" s="2">
+      <c r="T310">
+        <v>1</v>
+      </c>
+      <c r="U310" s="12">
+        <v>54.52</v>
+      </c>
+    </row>
+    <row r="311" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N311" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O311" cm="1">
         <f t="array" ref="O311">INDEX($F$6:$F$68, INT((ROWS(O$6:O311)-1)/5)+1)</f>
@@ -11783,12 +12550,17 @@
         <f t="array" ref="S311">INDEX($I$6:$I$68, INT((ROWS(S$6:S311)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U311" s="12"/>
-    </row>
-    <row r="312" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N312" s="2">
+      <c r="T311">
+        <v>2</v>
+      </c>
+      <c r="U311" s="12">
+        <v>56.05</v>
+      </c>
+    </row>
+    <row r="312" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N312" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O312" cm="1">
         <f t="array" ref="O312">INDEX($F$6:$F$68, INT((ROWS(O$6:O312)-1)/5)+1)</f>
@@ -11810,12 +12582,17 @@
         <f t="array" ref="S312">INDEX($I$6:$I$68, INT((ROWS(S$6:S312)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U312" s="12"/>
-    </row>
-    <row r="313" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N313" s="2">
+      <c r="T312">
+        <v>2</v>
+      </c>
+      <c r="U312" s="12">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="313" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N313" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O313" cm="1">
         <f t="array" ref="O313">INDEX($F$6:$F$68, INT((ROWS(O$6:O313)-1)/5)+1)</f>
@@ -11837,12 +12614,20 @@
         <f t="array" ref="S313">INDEX($I$6:$I$68, INT((ROWS(S$6:S313)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U313" s="12"/>
-    </row>
-    <row r="314" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N314" s="2">
+      <c r="T313">
+        <v>2</v>
+      </c>
+      <c r="U313" s="12">
+        <v>57.42</v>
+      </c>
+      <c r="X313" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="314" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N314" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O314" cm="1">
         <f t="array" ref="O314">INDEX($F$6:$F$68, INT((ROWS(O$6:O314)-1)/5)+1)</f>
@@ -11864,12 +12649,20 @@
         <f t="array" ref="S314">INDEX($I$6:$I$68, INT((ROWS(S$6:S314)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U314" s="12"/>
-    </row>
-    <row r="315" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N315" s="2">
+      <c r="T314">
+        <v>2</v>
+      </c>
+      <c r="U314" s="12">
+        <v>57.42</v>
+      </c>
+      <c r="X314" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="315" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N315" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O315" cm="1">
         <f t="array" ref="O315">INDEX($F$6:$F$68, INT((ROWS(O$6:O315)-1)/5)+1)</f>
@@ -11891,12 +12684,20 @@
         <f t="array" ref="S315">INDEX($I$6:$I$68, INT((ROWS(S$6:S315)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U315" s="12"/>
-    </row>
-    <row r="316" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N316" s="2">
+      <c r="T315">
+        <v>2</v>
+      </c>
+      <c r="U315" s="12">
+        <v>57.42</v>
+      </c>
+      <c r="X315" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="316" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N316" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O316" cm="1">
         <f t="array" ref="O316">INDEX($F$6:$F$68, INT((ROWS(O$6:O316)-1)/5)+1)</f>
@@ -11918,12 +12719,17 @@
         <f t="array" ref="S316">INDEX($I$6:$I$68, INT((ROWS(S$6:S316)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U316" s="12"/>
-    </row>
-    <row r="317" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N317" s="2">
+      <c r="T316">
+        <v>3</v>
+      </c>
+      <c r="U316" s="12">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="317" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N317" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O317" cm="1">
         <f t="array" ref="O317">INDEX($F$6:$F$68, INT((ROWS(O$6:O317)-1)/5)+1)</f>
@@ -11945,12 +12751,17 @@
         <f t="array" ref="S317">INDEX($I$6:$I$68, INT((ROWS(S$6:S317)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U317" s="12"/>
-    </row>
-    <row r="318" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N318" s="2">
+      <c r="T317">
+        <v>3</v>
+      </c>
+      <c r="U317" s="12">
+        <v>45.03</v>
+      </c>
+    </row>
+    <row r="318" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N318" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O318" cm="1">
         <f t="array" ref="O318">INDEX($F$6:$F$68, INT((ROWS(O$6:O318)-1)/5)+1)</f>
@@ -11972,12 +12783,17 @@
         <f t="array" ref="S318">INDEX($I$6:$I$68, INT((ROWS(S$6:S318)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U318" s="12"/>
-    </row>
-    <row r="319" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N319" s="2">
+      <c r="T318">
+        <v>3</v>
+      </c>
+      <c r="U318" s="12">
+        <v>41.19</v>
+      </c>
+    </row>
+    <row r="319" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N319" s="2" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O319" cm="1">
         <f t="array" ref="O319">INDEX($F$6:$F$68, INT((ROWS(O$6:O319)-1)/5)+1)</f>
@@ -11999,12 +12815,17 @@
         <f t="array" ref="S319">INDEX($I$6:$I$68, INT((ROWS(S$6:S319)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="U319" s="12"/>
-    </row>
-    <row r="320" spans="14:21" x14ac:dyDescent="0.25">
-      <c r="N320" s="4">
+      <c r="T319">
+        <v>3</v>
+      </c>
+      <c r="U319" s="12">
+        <v>41.13</v>
+      </c>
+    </row>
+    <row r="320" spans="14:24" x14ac:dyDescent="0.25">
+      <c r="N320" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>ES</v>
       </c>
       <c r="O320" s="5" cm="1">
         <f t="array" ref="O320">INDEX($F$6:$F$68, INT((ROWS(O$6:O320)-1)/5)+1)</f>
@@ -12026,8 +12847,12 @@
         <f t="array" ref="S320">INDEX($I$6:$I$68, INT((ROWS(S$6:S320)-1)/5)+1)</f>
         <v>3</v>
       </c>
-      <c r="T320" s="5"/>
-      <c r="U320" s="13"/>
+      <c r="T320">
+        <v>3</v>
+      </c>
+      <c r="U320" s="13">
+        <v>41.12</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12036,39 +12861,34 @@
     <mergeCell ref="X1:AA2"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:I68 K6:K68">
-    <cfRule type="expression" dxfId="6" priority="6">
+  <conditionalFormatting sqref="E6:K68">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>MOD(ROUNDDOWN((ROW()-6)/3,0),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:S13 N69:U90 N91:T92 N93:U320 N15:S68 U66:U68 U15:U50 U11:U13 U6">
-    <cfRule type="expression" dxfId="5" priority="7">
+  <conditionalFormatting sqref="N6:T320">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>MOD(ROUNDDOWN((ROW()-6)/5,0),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N14:S14 U14:V14">
-    <cfRule type="expression" dxfId="4" priority="3">
+  <conditionalFormatting sqref="U6 U15:U50 U66:U90 U93:U320">
+    <cfRule type="expression" dxfId="3" priority="9">
       <formula>MOD(ROUNDDOWN((ROW()-6)/5,0),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U11">
-    <cfRule type="expression" dxfId="3" priority="4">
+  <conditionalFormatting sqref="U8:U13">
+    <cfRule type="expression" dxfId="2" priority="6">
+      <formula>MOD(ROUNDDOWN((ROW()-6)/5,0),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U14:V14">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>MOD(ROUNDDOWN((ROW()-6)/5,0),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W113:W121">
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>MOD(ROUNDDOWN((ROW()-6)/5,0),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J68">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>MOD(ROUNDDOWN((ROW()-6)/3,0),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T6:T68">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>MOD(ROUNDDOWN((ROW()-6)/3,0),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12101,7 +12921,7 @@
   <sheetData>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -12109,10 +12929,10 @@
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -12120,7 +12940,7 @@
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -12128,103 +12948,103 @@
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="M6" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="M7" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="V7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
       </c>
       <c r="G9" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="M9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="O9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="P9" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="Q9" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="R9" t="s">
         <v>6</v>
       </c>
       <c r="V9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="L10" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="N10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="O10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="P10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="Q10" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="R10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
@@ -12659,7 +13479,7 @@
         <v>4</v>
       </c>
       <c r="K34" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" spans="3:15" x14ac:dyDescent="0.25">
@@ -12689,7 +13509,7 @@
         <v>8.5416666666666669E-2</v>
       </c>
       <c r="N35" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="O35">
         <f>CORREL(C11:C73,E11:E73)</f>
@@ -12766,7 +13586,7 @@
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="3:15" x14ac:dyDescent="0.25">
@@ -12787,7 +13607,7 @@
         <v>9</v>
       </c>
       <c r="K39" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="3:15" x14ac:dyDescent="0.25">
@@ -12808,7 +13628,7 @@
         <v>16</v>
       </c>
       <c r="K40" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="3:15" x14ac:dyDescent="0.25">
@@ -12829,7 +13649,7 @@
         <v>4</v>
       </c>
       <c r="K41" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="3:15" x14ac:dyDescent="0.25">
@@ -12850,7 +13670,7 @@
         <v>9</v>
       </c>
       <c r="K42" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="3:15" x14ac:dyDescent="0.25">
@@ -12871,7 +13691,7 @@
         <v>16</v>
       </c>
       <c r="K43" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="3:15" x14ac:dyDescent="0.25">
@@ -12892,7 +13712,7 @@
         <v>4</v>
       </c>
       <c r="K44" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="3:15" x14ac:dyDescent="0.25">
@@ -12913,7 +13733,7 @@
         <v>9</v>
       </c>
       <c r="K45" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="3:15" x14ac:dyDescent="0.25">
@@ -12970,7 +13790,7 @@
         <v>27</v>
       </c>
       <c r="K48" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="3:13" x14ac:dyDescent="0.25">
@@ -12991,7 +13811,7 @@
         <v>64</v>
       </c>
       <c r="K49" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" spans="3:13" x14ac:dyDescent="0.25">
@@ -13012,7 +13832,7 @@
         <v>8</v>
       </c>
       <c r="K50" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="51" spans="3:13" x14ac:dyDescent="0.25">
@@ -13033,7 +13853,7 @@
         <v>27</v>
       </c>
       <c r="K51" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="3:13" x14ac:dyDescent="0.25">
@@ -13054,7 +13874,7 @@
         <v>64</v>
       </c>
       <c r="K52" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="3:13" x14ac:dyDescent="0.25">
@@ -13129,7 +13949,7 @@
         <v>2</v>
       </c>
       <c r="L56" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="M56" t="s">
         <v>6</v>
@@ -13156,7 +13976,7 @@
         <v>1</v>
       </c>
       <c r="L57" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="M57">
         <v>1</v>
@@ -13183,7 +14003,7 @@
         <v>2</v>
       </c>
       <c r="L58" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="M58">
         <v>3</v>
@@ -13210,7 +14030,7 @@
         <v>3</v>
       </c>
       <c r="L59" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="M59">
         <v>3</v>
@@ -13536,21 +14356,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D707A1FFD900984DA43D6BF4AF7BE639" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="82a7a6aab175811d53c50c6095ba9899">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="418a5de5-9fd6-4eb7-9ae8-c174d6a3ca44" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="267367cbe5ea6f9eb0df44a21305574c" ns2:_="">
     <xsd:import namespace="418a5de5-9fd6-4eb7-9ae8-c174d6a3ca44"/>
@@ -13688,24 +14493,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECBB0E36-C83F-433A-89E2-B86DF40F23B7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4FE76C1-CDC6-4436-908E-D0E0AC210158}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2B8C8A5-5A5B-489F-B271-2734D641A242}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13721,4 +14524,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4FE76C1-CDC6-4436-908E-D0E0AC210158}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECBB0E36-C83F-433A-89E2-B86DF40F23B7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>